<commit_message>
DSM completed and tested
DSM successfully implemented and tested, manually and automatically within a test network
</commit_message>
<xml_diff>
--- a/data/Fertig - 1.a_MS_misch_base/1.a_MS_misch_grid-reduced/Power_DSM_Ramping.xlsx
+++ b/data/Fertig - 1.a_MS_misch_base/1.a_MS_misch_grid-reduced/Power_DSM_Ramping.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tom\Tu Graz\Masterarbeit\Git\LEGO-Pyomo\data\Fertig - 1.a_MS_misch_base\1.a_MS_misch_grid-reduced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3470F267-1037-45EF-B39F-00A79FB1D620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31ED4DE4-7360-48B5-9B52-DA66E247CCD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioA" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1737,7 +1750,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="23">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G10" s="13">
         <v>1</v>
@@ -1776,7 +1789,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="23">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G11" s="13">
         <v>2</v>

</xml_diff>